<commit_message>
supplier changes and purchase order changes
</commit_message>
<xml_diff>
--- a/public/files/purchase_order_export.xlsx
+++ b/public/files/purchase_order_export.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -43,6 +43,9 @@
     <t xml:space="preserve">Qty</t>
   </si>
   <si>
+    <t xml:space="preserve">Order By</t>
+  </si>
+  <si>
     <t xml:space="preserve">INI101</t>
   </si>
   <si>
@@ -55,6 +58,9 @@
     <t xml:space="preserve">ABG76868</t>
   </si>
   <si>
+    <t xml:space="preserve">PR Admin</t>
+  </si>
+  <si>
     <t xml:space="preserve">INI102</t>
   </si>
   <si>
@@ -67,6 +73,9 @@
     <t xml:space="preserve">ABG768345</t>
   </si>
   <si>
+    <t xml:space="preserve">Harvi Jivani</t>
+  </si>
+  <si>
     <t xml:space="preserve">INI103</t>
   </si>
   <si>
@@ -79,6 +88,9 @@
     <t xml:space="preserve">ABG743345</t>
   </si>
   <si>
+    <t xml:space="preserve">Denisha Rokad</t>
+  </si>
+  <si>
     <t xml:space="preserve">INI104</t>
   </si>
   <si>
@@ -89,6 +101,9 @@
   </si>
   <si>
     <t xml:space="preserve">ABG767345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Novok</t>
   </si>
 </sst>
 </file>
@@ -98,7 +113,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,6 +139,14 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -178,7 +201,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -192,6 +215,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -216,15 +243,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>177120</xdr:colOff>
+      <xdr:colOff>177480</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>143280</xdr:rowOff>
+      <xdr:rowOff>143640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>596880</xdr:colOff>
+      <xdr:colOff>596520</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>686520</xdr:rowOff>
+      <xdr:rowOff>686160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -237,8 +264,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="21464400">
-          <a:off x="977400" y="333360"/>
-          <a:ext cx="419760" cy="543240"/>
+          <a:off x="977760" y="333720"/>
+          <a:ext cx="419040" cy="542520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -260,9 +287,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>433440</xdr:colOff>
+      <xdr:colOff>432720</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>416880</xdr:rowOff>
+      <xdr:rowOff>416160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -276,7 +303,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="885240" y="1036080"/>
-          <a:ext cx="348480" cy="320040"/>
+          <a:ext cx="347760" cy="319320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -298,9 +325,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>538560</xdr:colOff>
+      <xdr:colOff>537840</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>416880</xdr:rowOff>
+      <xdr:rowOff>416160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -314,7 +341,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="885600" y="1797840"/>
-          <a:ext cx="453240" cy="320040"/>
+          <a:ext cx="452520" cy="319320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -336,9 +363,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>335520</xdr:colOff>
+      <xdr:colOff>334800</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>318600</xdr:rowOff>
+      <xdr:rowOff>317880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -352,7 +379,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="796680" y="2760840"/>
-          <a:ext cx="339120" cy="320040"/>
+          <a:ext cx="338400" cy="319320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -555,7 +582,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="11" style="1" width="15"/>
@@ -583,144 +610,158 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1"/>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="58.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="E2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
       <c r="Y2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="D3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>279.99</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
+      <c r="H3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
       <c r="Y3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="83.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
+      <c r="H4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
       <c r="Y4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="47" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="3" t="n">
+      <c r="A5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
+      <c r="H5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
inventory overview and max stock in product
</commit_message>
<xml_diff>
--- a/public/files/purchase_order_export.xlsx
+++ b/public/files/purchase_order_export.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t xml:space="preserve">Order By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum Stock </t>
   </si>
   <si>
     <t xml:space="preserve">INI101</t>
@@ -113,7 +116,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -152,6 +155,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -201,7 +211,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -219,6 +229,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -249,9 +263,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>596520</xdr:colOff>
+      <xdr:colOff>596160</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>686160</xdr:rowOff>
+      <xdr:rowOff>685800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -264,8 +278,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm rot="21464400">
-          <a:off x="977760" y="333720"/>
-          <a:ext cx="419040" cy="542520"/>
+          <a:off x="977760" y="334080"/>
+          <a:ext cx="418680" cy="542160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -287,9 +301,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>432720</xdr:colOff>
+      <xdr:colOff>432360</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>416160</xdr:rowOff>
+      <xdr:rowOff>415800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -303,7 +317,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="885240" y="1036080"/>
-          <a:ext cx="347760" cy="319320"/>
+          <a:ext cx="347400" cy="318960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -325,9 +339,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>537840</xdr:colOff>
+      <xdr:colOff>537480</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>416160</xdr:rowOff>
+      <xdr:rowOff>415800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -341,7 +355,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="885600" y="1797840"/>
-          <a:ext cx="452520" cy="319320"/>
+          <a:ext cx="452160" cy="318960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -363,9 +377,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>334800</xdr:colOff>
+      <xdr:colOff>334440</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>317880</xdr:rowOff>
+      <xdr:rowOff>317520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -379,7 +393,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="796680" y="2760840"/>
-          <a:ext cx="338400" cy="319320"/>
+          <a:ext cx="338040" cy="318960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -583,7 +597,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="11" style="1" width="15"/>
   </cols>
@@ -613,155 +627,169 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1"/>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="58.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="E2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <v>3</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
+      <c r="J2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+      <c r="X2" s="5"/>
       <c r="Y2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="E3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="5" t="n">
         <v>279.99</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>2</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
+        <v>18</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+      <c r="X3" s="5"/>
       <c r="Y3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="83.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>4</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="5"/>
       <c r="Y4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="47" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>5</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
+        <v>28</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+      <c r="X5" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>